<commit_message>
changes in ears excel report
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>FloorWalk</t>
   </si>
@@ -31,33 +31,21 @@
     <t>15-03-2017</t>
   </si>
   <si>
-    <t>Staff Names</t>
-  </si>
-  <si>
     <t>Place</t>
   </si>
   <si>
     <t>Showroom 3</t>
   </si>
   <si>
-    <t>Bowling</t>
-  </si>
-  <si>
     <t>Audit Time</t>
   </si>
   <si>
-    <t>Tele Operator</t>
-  </si>
-  <si>
     <t>Audit Score</t>
   </si>
   <si>
     <t>72%</t>
   </si>
   <si>
-    <t>Restaurant</t>
-  </si>
-  <si>
     <t>Points Lost</t>
   </si>
   <si>
@@ -76,37 +64,37 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Need Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff enquire about your purpose of visit?</t>
+  </si>
+  <si>
+    <t>Was the staff suggestive and interactive during displaying products?</t>
+  </si>
+  <si>
     <t>Entrance</t>
   </si>
   <si>
     <t>Was there ample parking space for visitors?</t>
   </si>
   <si>
-    <t>Need Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff enquire about your purpose of visit?</t>
-  </si>
-  <si>
-    <t>Was the staff suggestive and interactive during displaying products?</t>
+    <t>Selling and Recommendation skills</t>
+  </si>
+  <si>
+    <t>Did the staff ask for your budget before starting to show products?</t>
+  </si>
+  <si>
+    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
+  </si>
+  <si>
+    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
   <si>
     <t>Staff Analysis</t>
   </si>
   <si>
     <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
-  </si>
-  <si>
-    <t>Selling and Recommendation skills</t>
-  </si>
-  <si>
-    <t>Did the staff ask for your budget before starting to show products?</t>
-  </si>
-  <si>
-    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
-  </si>
-  <si>
-    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
 </sst>
 </file>
@@ -577,78 +565,70 @@
         <v>4</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -660,7 +640,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -669,34 +649,34 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="B12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
         <v>1</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -705,10 +685,10 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -720,7 +700,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -729,22 +709,22 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>3</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
         <v>1</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
@@ -755,20 +735,20 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="B18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
         <v>1</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -781,9 +761,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated snapshot of ears excel report
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -64,6 +64,12 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Entrance</t>
+  </si>
+  <si>
+    <t>Was there ample parking space for visitors?</t>
+  </si>
+  <si>
     <t>Need Analysis</t>
   </si>
   <si>
@@ -73,10 +79,10 @@
     <t>Was the staff suggestive and interactive during displaying products?</t>
   </si>
   <si>
-    <t>Entrance</t>
-  </si>
-  <si>
-    <t>Was there ample parking space for visitors?</t>
+    <t>Staff Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
   </si>
   <si>
     <t>Selling and Recommendation skills</t>
@@ -89,12 +95,6 @@
   </si>
   <si>
     <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
-  </si>
-  <si>
-    <t>Staff Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
   </si>
 </sst>
 </file>
@@ -625,7 +625,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>16</v>
@@ -649,27 +649,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -685,7 +685,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>21</v>
@@ -709,15 +709,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>1</v>
-      </c>
-      <c r="B16" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -735,13 +735,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -761,9 +761,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
code for pm comment
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -64,37 +64,37 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Need Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff enquire about your purpose of visit?</t>
+  </si>
+  <si>
+    <t>Was the staff suggestive and interactive during displaying products?</t>
+  </si>
+  <si>
     <t>Entrance</t>
   </si>
   <si>
     <t>Was there ample parking space for visitors?</t>
   </si>
   <si>
-    <t>Need Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff enquire about your purpose of visit?</t>
-  </si>
-  <si>
-    <t>Was the staff suggestive and interactive during displaying products?</t>
+    <t>Selling and Recommendation skills</t>
+  </si>
+  <si>
+    <t>Did the staff ask for your budget before starting to show products?</t>
+  </si>
+  <si>
+    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
+  </si>
+  <si>
+    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
   <si>
     <t>Staff Analysis</t>
   </si>
   <si>
     <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
-  </si>
-  <si>
-    <t>Selling and Recommendation skills</t>
-  </si>
-  <si>
-    <t>Did the staff ask for your budget before starting to show products?</t>
-  </si>
-  <si>
-    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
-  </si>
-  <si>
-    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
 </sst>
 </file>
@@ -625,7 +625,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>16</v>
@@ -649,27 +649,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -685,7 +685,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>21</v>
@@ -709,15 +709,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>3</v>
-      </c>
-      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -735,13 +735,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -761,9 +761,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added button code in fiat assign email, create ears report xlsx
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -64,37 +64,37 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Need Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff enquire about your purpose of visit?</t>
+  </si>
+  <si>
+    <t>Was the staff suggestive and interactive during displaying products?</t>
+  </si>
+  <si>
     <t>Entrance</t>
   </si>
   <si>
     <t>Was there ample parking space for visitors?</t>
   </si>
   <si>
-    <t>Need Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff enquire about your purpose of visit?</t>
-  </si>
-  <si>
-    <t>Was the staff suggestive and interactive during displaying products?</t>
+    <t>Selling and Recommendation skills</t>
+  </si>
+  <si>
+    <t>Did the staff ask for your budget before starting to show products?</t>
+  </si>
+  <si>
+    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
+  </si>
+  <si>
+    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
   <si>
     <t>Staff Analysis</t>
   </si>
   <si>
     <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
-  </si>
-  <si>
-    <t>Selling and Recommendation skills</t>
-  </si>
-  <si>
-    <t>Did the staff ask for your budget before starting to show products?</t>
-  </si>
-  <si>
-    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
-  </si>
-  <si>
-    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
 </sst>
 </file>
@@ -625,7 +625,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>16</v>
@@ -649,27 +649,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -685,7 +685,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>21</v>
@@ -709,15 +709,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>3</v>
-      </c>
-      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -735,13 +735,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -761,9 +761,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changes in ears excdel code
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>FloorWalk</t>
   </si>
@@ -31,19 +31,31 @@
     <t>15-03-2017</t>
   </si>
   <si>
+    <t>Staff Names</t>
+  </si>
+  <si>
     <t>Place</t>
   </si>
   <si>
     <t>Showroom 3</t>
   </si>
   <si>
+    <t>Bowling</t>
+  </si>
+  <si>
     <t>Audit Time</t>
   </si>
   <si>
+    <t>Tele Operator</t>
+  </si>
+  <si>
     <t>Audit Score</t>
   </si>
   <si>
     <t>72%</t>
+  </si>
+  <si>
+    <t>Restaurant</t>
   </si>
   <si>
     <t>Points Lost</t>
@@ -565,62 +577,70 @@
         <v>4</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
@@ -628,7 +648,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -640,7 +660,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -652,7 +672,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -664,7 +684,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -676,7 +696,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -688,7 +708,7 @@
         <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -700,7 +720,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -712,7 +732,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
@@ -724,7 +744,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
@@ -736,7 +756,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -748,7 +768,7 @@
         <v>1</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>

</xml_diff>

<commit_message>
update ears xlsx report
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -76,6 +76,12 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Entrance</t>
+  </si>
+  <si>
+    <t>Was there ample parking space for visitors?</t>
+  </si>
+  <si>
     <t>Need Analysis</t>
   </si>
   <si>
@@ -85,10 +91,10 @@
     <t>Was the staff suggestive and interactive during displaying products?</t>
   </si>
   <si>
-    <t>Entrance</t>
-  </si>
-  <si>
-    <t>Was there ample parking space for visitors?</t>
+    <t>Staff Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
   </si>
   <si>
     <t>Selling and Recommendation skills</t>
@@ -101,12 +107,6 @@
   </si>
   <si>
     <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
-  </si>
-  <si>
-    <t>Staff Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
   </si>
 </sst>
 </file>
@@ -645,7 +645,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>20</v>
@@ -669,27 +669,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -705,7 +705,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>25</v>
@@ -729,15 +729,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>1</v>
-      </c>
-      <c r="B16" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -755,13 +755,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -781,9 +781,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B11:F11"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B16:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update ears excel file
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -76,37 +76,37 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Need Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff enquire about your purpose of visit?</t>
+  </si>
+  <si>
+    <t>Was the staff suggestive and interactive during displaying products?</t>
+  </si>
+  <si>
     <t>Entrance</t>
   </si>
   <si>
     <t>Was there ample parking space for visitors?</t>
   </si>
   <si>
-    <t>Need Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff enquire about your purpose of visit?</t>
-  </si>
-  <si>
-    <t>Was the staff suggestive and interactive during displaying products?</t>
+    <t>Selling and Recommendation skills</t>
+  </si>
+  <si>
+    <t>Did the staff ask for your budget before starting to show products?</t>
+  </si>
+  <si>
+    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
+  </si>
+  <si>
+    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
   <si>
     <t>Staff Analysis</t>
   </si>
   <si>
     <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
-  </si>
-  <si>
-    <t>Selling and Recommendation skills</t>
-  </si>
-  <si>
-    <t>Did the staff ask for your budget before starting to show products?</t>
-  </si>
-  <si>
-    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
-  </si>
-  <si>
-    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
 </sst>
 </file>
@@ -645,7 +645,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>20</v>
@@ -669,27 +669,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -705,7 +705,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>25</v>
@@ -729,15 +729,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>3</v>
-      </c>
-      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -755,13 +755,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -781,9 +781,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
showing one audit cycle also in proof comparison, changed failed text to rejected in failed mail
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -76,37 +76,37 @@
     <t>Date Committed</t>
   </si>
   <si>
+    <t>Need Analysis</t>
+  </si>
+  <si>
+    <t>Did the staff enquire about your purpose of visit?</t>
+  </si>
+  <si>
+    <t>Was the staff suggestive and interactive during displaying products?</t>
+  </si>
+  <si>
     <t>Entrance</t>
   </si>
   <si>
     <t>Was there ample parking space for visitors?</t>
   </si>
   <si>
-    <t>Need Analysis</t>
-  </si>
-  <si>
-    <t>Did the staff enquire about your purpose of visit?</t>
-  </si>
-  <si>
-    <t>Was the staff suggestive and interactive during displaying products?</t>
+    <t>Selling and Recommendation skills</t>
+  </si>
+  <si>
+    <t>Did the staff ask for your budget before starting to show products?</t>
+  </si>
+  <si>
+    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
+  </si>
+  <si>
+    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
   <si>
     <t>Staff Analysis</t>
   </si>
   <si>
     <t>Did the staff member seemed energetic and enthusiastic while interacting with you?</t>
-  </si>
-  <si>
-    <t>Selling and Recommendation skills</t>
-  </si>
-  <si>
-    <t>Did the staff ask for your budget before starting to show products?</t>
-  </si>
-  <si>
-    <t>Did the staff member insisted upon taking a trial of the chosen product?</t>
-  </si>
-  <si>
-    <t>Were you satisfied with the amount of effort put in by the staff member to make that deal happen?</t>
   </si>
 </sst>
 </file>
@@ -645,7 +645,7 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>20</v>
@@ -669,27 +669,27 @@
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="5">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="5">
@@ -705,7 +705,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>25</v>
@@ -729,15 +729,15 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="5">
-        <v>3</v>
-      </c>
-      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="5">
@@ -755,13 +755,13 @@
       <c r="A18" s="5">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1">
       <c r="A19" s="5">
@@ -781,9 +781,9 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
code for auditor dob year range(min 15 and max 80), auditor rating mandatory for manager, changes in test_ears_excel file
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/generate_ears_report_for_clientuser_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>FloorWalk</t>
   </si>
@@ -31,31 +31,19 @@
     <t>15-03-2017</t>
   </si>
   <si>
-    <t>Staff Names</t>
-  </si>
-  <si>
     <t>Place</t>
   </si>
   <si>
     <t>Showroom 3</t>
   </si>
   <si>
-    <t>Bowling</t>
-  </si>
-  <si>
     <t>Audit Time</t>
   </si>
   <si>
-    <t>Tele Operator</t>
-  </si>
-  <si>
     <t>Audit Score</t>
   </si>
   <si>
     <t>72%</t>
-  </si>
-  <si>
-    <t>Restaurant</t>
   </si>
   <si>
     <t>Points Lost</t>
@@ -577,70 +565,62 @@
         <v>4</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
@@ -648,7 +628,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -660,7 +640,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -672,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -684,7 +664,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -696,7 +676,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -708,7 +688,7 @@
         <v>3</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -720,7 +700,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -732,7 +712,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
@@ -744,7 +724,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
@@ -756,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -768,7 +748,7 @@
         <v>1</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>

</xml_diff>